<commit_message>
chore: back up gameplay refactors and commander 10Hz profiling evidence
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeBuildings.xlsx
+++ b/data/Excel/GuLiStrikeBuildings.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>id</t>
   </si>
@@ -209,6 +209,9 @@
   </si>
   <si>
     <t>4,5,6</t>
+  </si>
+  <si>
+    <t>TransitFieldId</t>
   </si>
 </sst>
 </file>
@@ -610,7 +613,7 @@
         <v>32</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="AC1" s="1" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
chore: back up scale 0.2 gameplay, ship art, warning UI and lighting updates
Include current project code, configuration, data sources, authored assets, production tools and verification records. Keep marketplace pine sources, copied source geometry, original backups, generated tooling and existing local-only maps excluded; store delivery archives with Git LFS.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeBuildings.xlsx
+++ b/data/Excel/GuLiStrikeBuildings.xlsx
@@ -832,31 +832,31 @@
         <v>40</v>
       </c>
       <c r="I4">
-        <v>1259.73111</v>
+        <v>251.946222</v>
       </c>
       <c r="J4">
-        <v>1364.374146</v>
+        <v>272.8748292</v>
       </c>
       <c r="K4">
-        <v>1760.383118</v>
+        <v>352.0766236</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
-        <v>-24.28981</v>
+        <v>-4.857962</v>
       </c>
       <c r="N4">
         <v>0</v>
       </c>
       <c r="O4">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="P4">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="Q4">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="R4">
         <v>2000</v>
@@ -903,13 +903,13 @@
         <v>44</v>
       </c>
       <c r="I5">
-        <v>967.89624</v>
+        <v>193.579248</v>
       </c>
       <c r="J5">
-        <v>1933.390137</v>
+        <v>386.6780274</v>
       </c>
       <c r="K5">
-        <v>837.594452</v>
+        <v>167.5188904</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -918,16 +918,16 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>3.978149</v>
+        <v>0.7956298</v>
       </c>
       <c r="O5">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="P5">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="R5">
         <v>1500</v>
@@ -974,31 +974,31 @@
         <v>48</v>
       </c>
       <c r="I6">
-        <v>3551.543213</v>
+        <v>710.3086426</v>
       </c>
       <c r="J6">
-        <v>3309.902588</v>
+        <v>661.9805176</v>
       </c>
       <c r="K6">
-        <v>15000</v>
+        <v>3000</v>
       </c>
       <c r="L6">
-        <v>10.589355</v>
+        <v>2.117871</v>
       </c>
       <c r="M6">
-        <v>-252.585938</v>
+        <v>-50.5171876</v>
       </c>
       <c r="N6">
         <v>0</v>
       </c>
       <c r="O6">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="P6">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="Q6">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="R6">
         <v>5000</v>
@@ -1045,13 +1045,13 @@
         <v>52</v>
       </c>
       <c r="I7">
-        <v>2000</v>
+        <v>400</v>
       </c>
       <c r="J7">
-        <v>1500</v>
+        <v>300</v>
       </c>
       <c r="K7">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -1060,16 +1060,16 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="O7">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="P7">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="Q7">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="R7">
         <v>2000</v>
@@ -1125,16 +1125,16 @@
         <v>56</v>
       </c>
       <c r="I8">
-        <v>1525.43503</v>
+        <v>305.087006</v>
       </c>
       <c r="J8">
-        <v>1726.4402</v>
+        <v>345.28804</v>
       </c>
       <c r="K8">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="L8">
-        <v>234.56497</v>
+        <v>46.912994</v>
       </c>
       <c r="M8">
         <v>0</v>
@@ -1143,13 +1143,13 @@
         <v>0</v>
       </c>
       <c r="O8">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="P8">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q8">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="R8">
         <v>2000</v>
@@ -1170,7 +1170,7 @@
         <v>10</v>
       </c>
       <c r="AC8">
-        <v>20000</v>
+        <v>4000</v>
       </c>
       <c r="AD8">
         <v>20</v>
@@ -1202,13 +1202,13 @@
         <v>52</v>
       </c>
       <c r="I9">
-        <v>3000</v>
+        <v>600</v>
       </c>
       <c r="J9">
-        <v>3250</v>
+        <v>650</v>
       </c>
       <c r="K9">
-        <v>2000</v>
+        <v>400</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -1217,16 +1217,16 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>2000</v>
+        <v>400</v>
       </c>
       <c r="O9">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="P9">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="Q9">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="R9">
         <v>3000</v>
@@ -1273,13 +1273,13 @@
         <v>63</v>
       </c>
       <c r="I10">
-        <v>1500</v>
+        <v>300</v>
       </c>
       <c r="J10">
-        <v>1500</v>
+        <v>300</v>
       </c>
       <c r="K10">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -1288,16 +1288,16 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="O10">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="P10">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="Q10">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="R10">
         <v>1</v>

</xml_diff>

<commit_message>
chore: sync project changes and archive approved SSF buildings
Include all current project source, data, assets, art sources, and progress records. Preserve approved SSF deliverables and audit the cleanup of session-generated temporary files.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeBuildings.xlsx
+++ b/data/Excel/GuLiStrikeBuildings.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>id</t>
   </si>
@@ -212,6 +212,27 @@
   </si>
   <si>
     <t>TransitFieldId</t>
+  </si>
+  <si>
+    <t>CompletionUnitTypeId</t>
+  </si>
+  <si>
+    <t>BiZhiMaoConstruction</t>
+  </si>
+  <si>
+    <t>仅己方工程车贡献60工作量；完工原位转兵种ID6；人口预留1</t>
+  </si>
+  <si>
+    <t>彼之矛</t>
+  </si>
+  <si>
+    <t>巨型重炮工地：60蓝、30红、1人口；完工展开待机，等待指令。</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Commander/Units/BiZhiMao/Meshes/SM_BiZhiMao_Construction.SM_BiZhiMao_Construction</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Commander/Units/BiZhiMao/LOD_3Tier_v1/Meshes/SM_BiZhiMao_Construction.SM_BiZhiMao_Construction</t>
   </si>
 </sst>
 </file>
@@ -621,6 +642,9 @@
       <c r="AD1" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="AE1" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -713,6 +737,9 @@
       <c r="AD2" t="s">
         <v>14</v>
       </c>
+      <c r="AE2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -805,6 +832,9 @@
       <c r="AD3" t="s">
         <v>6</v>
       </c>
+      <c r="AE3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -876,6 +906,9 @@
       <c r="W4">
         <v>10</v>
       </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -946,6 +979,9 @@
       </c>
       <c r="W5">
         <v>10</v>
+      </c>
+      <c r="AE5">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1018,6 +1054,9 @@
       <c r="W6">
         <v>10</v>
       </c>
+      <c r="AE6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -1098,6 +1137,9 @@
       <c r="Z7">
         <v>24</v>
       </c>
+      <c r="AE7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -1175,6 +1217,9 @@
       <c r="AD8">
         <v>20</v>
       </c>
+      <c r="AE8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -1245,6 +1290,9 @@
       </c>
       <c r="W9">
         <v>10</v>
+      </c>
+      <c r="AE9">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1323,6 +1371,101 @@
       <c r="AB10">
         <v>2001</v>
       </c>
+      <c r="AE10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11">
+        <v>6</v>
+      </c>
+      <c r="E11">
+        <v>7</v>
+      </c>
+      <c r="F11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" t="s">
+        <v>70</v>
+      </c>
+      <c r="H11" t="s">
+        <v>72</v>
+      </c>
+      <c r="I11">
+        <v>1629.010009765625</v>
+      </c>
+      <c r="J11">
+        <v>921.9329833984375</v>
+      </c>
+      <c r="K11">
+        <v>690.5267333984375</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>2</v>
+      </c>
+      <c r="P11">
+        <v>2</v>
+      </c>
+      <c r="Q11">
+        <v>2</v>
+      </c>
+      <c r="R11">
+        <v>1000</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>1</v>
+      </c>
+      <c r="U11">
+        <v>60</v>
+      </c>
+      <c r="V11">
+        <v>30</v>
+      </c>
+      <c r="W11">
+        <v>60</v>
+      </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
+        <v>0</v>
+      </c>
+      <c r="AC11">
+        <v>0</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+      <c r="AE11">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
feat: unify model catalog, local team colors and scene UI
Register gameplay model IDs, resource bindings and mutable material regions through Excel and DataTables. Apply local friendly blue and enemy palettes to shared approved assets, including Sweeper orange UV regions, and draw environment-isolated scene UI with 20 cm rings. Preserve art approval history and runtime evidence; update documentation and remove session-only backups and scratch files.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeBuildings.xlsx
+++ b/data/Excel/GuLiStrikeBuildings.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
   <si>
     <t>id</t>
   </si>
@@ -233,6 +233,159 @@
   </si>
   <si>
     <t>/Game/GuLiStrike/Commander/Units/BiZhiMao/LOD_3Tier_v1/Meshes/SM_BiZhiMao_Construction.SM_BiZhiMao_Construction</t>
+  </si>
+  <si>
+    <t>ModelId</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>251.946222</t>
+  </si>
+  <si>
+    <t>272.8748292</t>
+  </si>
+  <si>
+    <t>352.0766236</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>-4.857962</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
+  <si>
+    <t>2000</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>193.579248</t>
+  </si>
+  <si>
+    <t>386.6780274</t>
+  </si>
+  <si>
+    <t>167.5188904</t>
+  </si>
+  <si>
+    <t>0.7956298</t>
+  </si>
+  <si>
+    <t>1500</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>710.3086426</t>
+  </si>
+  <si>
+    <t>661.9805176</t>
+  </si>
+  <si>
+    <t>3000</t>
+  </si>
+  <si>
+    <t>2.117871</t>
+  </si>
+  <si>
+    <t>-50.5171876</t>
+  </si>
+  <si>
+    <t>5000</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>305.087006</t>
+  </si>
+  <si>
+    <t>345.28804</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>46.912994</t>
+  </si>
+  <si>
+    <t>4000</t>
+  </si>
+  <si>
+    <t>600</t>
+  </si>
+  <si>
+    <t>650</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>2001</t>
+  </si>
+  <si>
+    <t>1629.010009765625</t>
+  </si>
+  <si>
+    <t>921.9329833984375</t>
+  </si>
+  <si>
+    <t>690.5267333984375</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>60</t>
   </si>
 </sst>
 </file>
@@ -574,76 +727,76 @@
         <v>10</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AD1" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="AD1" t="s">
+        <v>66</v>
+      </c>
       <c r="AE1" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2">
@@ -669,7 +822,7 @@
         <v>4</v>
       </c>
       <c r="H2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I2" t="s">
         <v>14</v>
@@ -702,40 +855,40 @@
         <v>14</v>
       </c>
       <c r="S2" t="s">
+        <v>1</v>
+      </c>
+      <c r="T2" t="s">
+        <v>1</v>
+      </c>
+      <c r="U2" t="s">
+        <v>1</v>
+      </c>
+      <c r="V2" t="s">
         <v>14</v>
       </c>
-      <c r="T2" t="s">
-        <v>1</v>
-      </c>
-      <c r="U2" t="s">
-        <v>1</v>
-      </c>
-      <c r="V2" t="s">
-        <v>1</v>
-      </c>
       <c r="W2" t="s">
+        <v>1</v>
+      </c>
+      <c r="X2" t="s">
         <v>14</v>
       </c>
-      <c r="X2" t="s">
-        <v>1</v>
-      </c>
       <c r="Y2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB2" t="s">
         <v>14</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>4</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>1</v>
       </c>
       <c r="AC2" t="s">
         <v>14</v>
       </c>
       <c r="AD2" t="s">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AE2" t="s">
         <v>1</v>
@@ -773,7 +926,7 @@
         <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L3" t="s">
         <v>6</v>
@@ -782,7 +935,7 @@
         <v>6</v>
       </c>
       <c r="N3" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O3" t="s">
         <v>2</v>
@@ -794,7 +947,7 @@
         <v>2</v>
       </c>
       <c r="R3" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="S3" t="s">
         <v>6</v>
@@ -833,7 +986,7 @@
         <v>6</v>
       </c>
       <c r="AE3" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -858,26 +1011,26 @@
       <c r="G4" t="s">
         <v>39</v>
       </c>
-      <c r="H4" t="s">
-        <v>40</v>
+      <c r="H4">
+        <v>251.946222</v>
       </c>
       <c r="I4">
-        <v>251.946222</v>
+        <v>272.8748292</v>
       </c>
       <c r="J4">
-        <v>272.8748292</v>
+        <v>352.0766236</v>
       </c>
       <c r="K4">
-        <v>352.0766236</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>0</v>
+        <v>-4.857962</v>
       </c>
       <c r="M4">
-        <v>-4.857962</v>
+        <v>0</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="O4">
         <v>0.2</v>
@@ -886,28 +1039,49 @@
         <v>0.2</v>
       </c>
       <c r="Q4">
-        <v>0.2</v>
+        <v>2000</v>
       </c>
       <c r="R4">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="U4">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="V4">
-        <v>0</v>
-      </c>
-      <c r="W4">
         <v>10</v>
       </c>
+      <c r="W4" t="s">
+        <v>84</v>
+      </c>
+      <c r="X4" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>84</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>84</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>84</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
       <c r="AE4">
-        <v>0</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="5">
@@ -932,26 +1106,26 @@
       <c r="G5" t="s">
         <v>43</v>
       </c>
-      <c r="H5" t="s">
-        <v>44</v>
+      <c r="H5">
+        <v>193.579248</v>
       </c>
       <c r="I5">
-        <v>193.579248</v>
+        <v>386.6780274</v>
       </c>
       <c r="J5">
-        <v>386.6780274</v>
+        <v>167.5188904</v>
       </c>
       <c r="K5">
-        <v>167.5188904</v>
+        <v>0</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>0.7956298</v>
       </c>
       <c r="N5">
-        <v>0.7956298</v>
+        <v>0.2</v>
       </c>
       <c r="O5">
         <v>0.2</v>
@@ -960,28 +1134,49 @@
         <v>0.2</v>
       </c>
       <c r="Q5">
-        <v>0.2</v>
+        <v>1500</v>
       </c>
       <c r="R5">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
         <v>10</v>
       </c>
-      <c r="V5">
-        <v>0</v>
-      </c>
-      <c r="W5">
-        <v>10</v>
+      <c r="W5" t="s">
+        <v>84</v>
+      </c>
+      <c r="X5" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>84</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
       </c>
       <c r="AE5">
-        <v>0</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="6">
@@ -1006,26 +1201,26 @@
       <c r="G6" t="s">
         <v>47</v>
       </c>
-      <c r="H6" t="s">
-        <v>48</v>
+      <c r="H6">
+        <v>710.3086426</v>
       </c>
       <c r="I6">
-        <v>710.3086426</v>
+        <v>661.9805176</v>
       </c>
       <c r="J6">
-        <v>661.9805176</v>
+        <v>3000</v>
       </c>
       <c r="K6">
-        <v>3000</v>
+        <v>2.117871</v>
       </c>
       <c r="L6">
-        <v>2.117871</v>
+        <v>-50.5171876</v>
       </c>
       <c r="M6">
-        <v>-50.5171876</v>
+        <v>0</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="O6">
         <v>0.2</v>
@@ -1034,28 +1229,49 @@
         <v>0.2</v>
       </c>
       <c r="Q6">
-        <v>0.2</v>
+        <v>5000</v>
       </c>
       <c r="R6">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="U6">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="V6">
-        <v>0</v>
-      </c>
-      <c r="W6">
         <v>10</v>
       </c>
+      <c r="W6" t="s">
+        <v>84</v>
+      </c>
+      <c r="X6" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>84</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>84</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>84</v>
+      </c>
+      <c r="AD6">
+        <v>0</v>
+      </c>
       <c r="AE6">
-        <v>0</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="7">
@@ -1080,65 +1296,77 @@
       <c r="G7" t="s">
         <v>51</v>
       </c>
-      <c r="H7" t="s">
-        <v>52</v>
+      <c r="H7">
+        <v>400</v>
       </c>
       <c r="I7">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="J7">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
         <v>200</v>
       </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
       <c r="N7">
-        <v>200</v>
+        <v>8</v>
       </c>
       <c r="O7">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q7">
-        <v>4</v>
+        <v>2000</v>
       </c>
       <c r="R7">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="S7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T7">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="U7">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="V7">
         <v>10</v>
       </c>
       <c r="W7">
+        <v>1</v>
+      </c>
+      <c r="X7">
         <v>10</v>
       </c>
-      <c r="X7">
-        <v>1</v>
-      </c>
       <c r="Y7">
-        <v>10</v>
-      </c>
-      <c r="Z7">
         <v>24</v>
       </c>
+      <c r="Z7" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>84</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>84</v>
+      </c>
+      <c r="AD7">
+        <v>0</v>
+      </c>
       <c r="AE7">
-        <v>0</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="8">
@@ -1163,62 +1391,77 @@
       <c r="G8" t="s">
         <v>55</v>
       </c>
-      <c r="H8" t="s">
-        <v>56</v>
+      <c r="H8">
+        <v>305.087006</v>
       </c>
       <c r="I8">
-        <v>305.087006</v>
+        <v>345.28804</v>
       </c>
       <c r="J8">
-        <v>345.28804</v>
+        <v>500</v>
       </c>
       <c r="K8">
+        <v>46.912994</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>2</v>
+      </c>
+      <c r="O8">
+        <v>2</v>
+      </c>
+      <c r="P8">
+        <v>2</v>
+      </c>
+      <c r="Q8">
+        <v>2000</v>
+      </c>
+      <c r="R8">
         <v>500</v>
       </c>
-      <c r="L8">
-        <v>46.912994</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>0</v>
-      </c>
-      <c r="O8">
-        <v>2</v>
-      </c>
-      <c r="P8">
-        <v>2</v>
-      </c>
-      <c r="Q8">
-        <v>2</v>
-      </c>
-      <c r="R8">
-        <v>2000</v>
-      </c>
       <c r="S8">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="T8">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="U8">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="V8">
         <v>10</v>
       </c>
-      <c r="W8">
-        <v>10</v>
+      <c r="W8" t="s">
+        <v>84</v>
+      </c>
+      <c r="X8" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>84</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>84</v>
+      </c>
+      <c r="AB8">
+        <v>4000</v>
       </c>
       <c r="AC8">
-        <v>4000</v>
+        <v>20</v>
       </c>
       <c r="AD8">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="AE8">
-        <v>0</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="9">
@@ -1243,56 +1486,77 @@
       <c r="G9" t="s">
         <v>59</v>
       </c>
-      <c r="H9" t="s">
-        <v>52</v>
+      <c r="H9">
+        <v>600</v>
       </c>
       <c r="I9">
-        <v>600</v>
+        <v>650</v>
       </c>
       <c r="J9">
-        <v>650</v>
+        <v>400</v>
       </c>
       <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
         <v>400</v>
       </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
       <c r="N9">
-        <v>400</v>
+        <v>12</v>
       </c>
       <c r="O9">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P9">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="Q9">
-        <v>8</v>
+        <v>3000</v>
       </c>
       <c r="R9">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="S9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="U9">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="V9">
         <v>10</v>
       </c>
-      <c r="W9">
-        <v>10</v>
+      <c r="W9" t="s">
+        <v>84</v>
+      </c>
+      <c r="X9" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>84</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>84</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>84</v>
+      </c>
+      <c r="AD9">
+        <v>0</v>
       </c>
       <c r="AE9">
-        <v>0</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="10">
@@ -1317,38 +1581,38 @@
       <c r="G10" t="s">
         <v>62</v>
       </c>
-      <c r="H10" t="s">
-        <v>63</v>
+      <c r="H10">
+        <v>300</v>
       </c>
       <c r="I10">
         <v>300</v>
       </c>
       <c r="J10">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
         <v>500</v>
       </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
       <c r="N10">
-        <v>500</v>
+        <v>6</v>
       </c>
       <c r="O10">
         <v>6</v>
       </c>
       <c r="P10">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="Q10">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="R10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10">
         <v>0</v>
@@ -1362,17 +1626,32 @@
       <c r="V10">
         <v>0</v>
       </c>
-      <c r="W10">
-        <v>0</v>
-      </c>
-      <c r="AA10" t="s">
+      <c r="W10" t="s">
+        <v>84</v>
+      </c>
+      <c r="X10" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>84</v>
+      </c>
+      <c r="Z10" t="s">
         <v>64</v>
       </c>
-      <c r="AB10">
+      <c r="AA10">
         <v>2001</v>
       </c>
+      <c r="AB10" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>84</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
       <c r="AE10">
-        <v>0</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="11">
@@ -1397,17 +1676,17 @@
       <c r="G11" t="s">
         <v>70</v>
       </c>
-      <c r="H11" t="s">
-        <v>72</v>
+      <c r="H11">
+        <v>1629.010009765625</v>
       </c>
       <c r="I11">
-        <v>1629.010009765625</v>
+        <v>921.9329833984375</v>
       </c>
       <c r="J11">
-        <v>921.9329833984375</v>
+        <v>690.5267333984375</v>
       </c>
       <c r="K11">
-        <v>690.5267333984375</v>
+        <v>0</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1416,7 +1695,7 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O11">
         <v>2</v>
@@ -1425,25 +1704,25 @@
         <v>2</v>
       </c>
       <c r="Q11">
-        <v>2</v>
+        <v>1000</v>
       </c>
       <c r="R11">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="S11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T11">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="U11">
+        <v>30</v>
+      </c>
+      <c r="V11">
         <v>60</v>
       </c>
-      <c r="V11">
-        <v>30</v>
-      </c>
       <c r="W11">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="X11">
         <v>0</v>
@@ -1451,7 +1730,10 @@
       <c r="Y11">
         <v>0</v>
       </c>
-      <c r="Z11">
+      <c r="Z11" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA11">
         <v>0</v>
       </c>
       <c r="AB11">
@@ -1461,10 +1743,10 @@
         <v>0</v>
       </c>
       <c r="AD11">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE11">
-        <v>6</v>
+        <v>2008</v>
       </c>
     </row>
   </sheetData>

</xml_diff>